<commit_message>
feat: update project report and test results spreadsheet with new findings and formatting improvements
</commit_message>
<xml_diff>
--- a/Proyecto Final ADA-PCD Pruebas.xlsx
+++ b/Proyecto Final ADA-PCD Pruebas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\University\ada\Proyecto-ADA-2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAFCEAB5-B9E2-4AB6-923A-652802969269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15A67CC-5706-4E60-897B-185D11F1E52A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14880" yWindow="840" windowWidth="21375" windowHeight="19425" firstSheet="4" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="15225" yWindow="1185" windowWidth="21375" windowHeight="19425" firstSheet="1" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla" sheetId="14" r:id="rId1"/>
@@ -3880,18 +3880,6 @@
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -3918,6 +3906,18 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3947,12 +3947,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="6" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3988,7 +3982,25 @@
     <xf numFmtId="0" fontId="11" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3997,19 +4009,19 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -4031,18 +4043,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -36356,44 +36356,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.75">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="126" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="135" t="s">
         <v>177</v>
       </c>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="127" t="s">
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
+      <c r="F1" s="136" t="s">
         <v>377</v>
       </c>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="128" t="s">
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="137" t="s">
         <v>525</v>
       </c>
-      <c r="J1" s="128"/>
-      <c r="K1" s="128"/>
-      <c r="L1" s="129" t="s">
+      <c r="J1" s="137"/>
+      <c r="K1" s="137"/>
+      <c r="L1" s="125" t="s">
         <v>575</v>
       </c>
-      <c r="M1" s="130"/>
-      <c r="N1" s="131"/>
-      <c r="O1" s="132" t="s">
+      <c r="M1" s="126"/>
+      <c r="N1" s="127"/>
+      <c r="O1" s="128" t="s">
         <v>210</v>
       </c>
-      <c r="P1" s="133"/>
-      <c r="Q1" s="133"/>
-      <c r="R1" s="133"/>
-      <c r="S1" s="133"/>
-      <c r="T1" s="134"/>
+      <c r="P1" s="129"/>
+      <c r="Q1" s="129"/>
+      <c r="R1" s="129"/>
+      <c r="S1" s="129"/>
+      <c r="T1" s="130"/>
     </row>
     <row r="2" spans="1:20" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="13" t="s">
         <v>1</v>
       </c>
@@ -38550,11 +38550,11 @@
       </c>
     </row>
     <row r="53" spans="1:20" ht="18.75">
-      <c r="I53" s="135" t="s">
+      <c r="I53" s="131" t="s">
         <v>370</v>
       </c>
-      <c r="J53" s="135"/>
-      <c r="K53" s="135"/>
+      <c r="J53" s="131"/>
+      <c r="K53" s="131"/>
       <c r="L53" s="26"/>
       <c r="M53" s="45"/>
       <c r="N53" s="45"/>
@@ -38584,11 +38584,11 @@
       </c>
     </row>
     <row r="54" spans="1:20" ht="18.75">
-      <c r="I54" s="136" t="s">
+      <c r="I54" s="132" t="s">
         <v>371</v>
       </c>
-      <c r="J54" s="136"/>
-      <c r="K54" s="136"/>
+      <c r="J54" s="132"/>
+      <c r="K54" s="132"/>
       <c r="L54" s="27"/>
       <c r="M54" s="46"/>
       <c r="N54" s="46"/>
@@ -38618,11 +38618,11 @@
       </c>
     </row>
     <row r="55" spans="1:20" ht="18.75">
-      <c r="I55" s="137" t="s">
+      <c r="I55" s="133" t="s">
         <v>372</v>
       </c>
-      <c r="J55" s="137"/>
-      <c r="K55" s="137"/>
+      <c r="J55" s="133"/>
+      <c r="K55" s="133"/>
       <c r="L55" s="28"/>
       <c r="M55" s="47"/>
       <c r="N55" s="47"/>
@@ -38673,16 +38673,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="L1:N1"/>
     <mergeCell ref="O1:T1"/>
     <mergeCell ref="I53:K53"/>
     <mergeCell ref="I54:K54"/>
     <mergeCell ref="I55:K55"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="I1:K1"/>
   </mergeCells>
   <conditionalFormatting sqref="O1:O52 O56:O1048576">
     <cfRule type="colorScale" priority="3">
@@ -38984,37 +38984,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.75">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="126" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="135" t="s">
         <v>177</v>
       </c>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="127" t="s">
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
+      <c r="F1" s="136" t="s">
         <v>377</v>
       </c>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="128" t="s">
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="137" t="s">
         <v>525</v>
       </c>
-      <c r="J1" s="128"/>
-      <c r="K1" s="128"/>
-      <c r="L1" s="132" t="s">
+      <c r="J1" s="137"/>
+      <c r="K1" s="137"/>
+      <c r="L1" s="128" t="s">
         <v>210</v>
       </c>
-      <c r="M1" s="133"/>
-      <c r="N1" s="133"/>
-      <c r="O1" s="133"/>
+      <c r="M1" s="129"/>
+      <c r="N1" s="129"/>
+      <c r="O1" s="129"/>
     </row>
     <row r="2" spans="1:15" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
@@ -41555,11 +41555,11 @@
       </c>
     </row>
     <row r="52" spans="1:15" ht="18.75">
-      <c r="I52" s="135" t="s">
+      <c r="I52" s="131" t="s">
         <v>370</v>
       </c>
-      <c r="J52" s="135"/>
-      <c r="K52" s="135"/>
+      <c r="J52" s="131"/>
+      <c r="K52" s="131"/>
       <c r="L52" s="18">
         <f>AVERAGE(L$3:L$51)</f>
         <v>7.6530612244897961E-2</v>
@@ -41578,11 +41578,11 @@
       </c>
     </row>
     <row r="53" spans="1:15" ht="18.75">
-      <c r="I53" s="136" t="s">
+      <c r="I53" s="132" t="s">
         <v>371</v>
       </c>
-      <c r="J53" s="136"/>
-      <c r="K53" s="136"/>
+      <c r="J53" s="132"/>
+      <c r="K53" s="132"/>
       <c r="L53" s="14">
         <f>MIN(L$3:L$51)</f>
         <v>0</v>
@@ -41601,11 +41601,11 @@
       </c>
     </row>
     <row r="54" spans="1:15" ht="18.75">
-      <c r="I54" s="137" t="s">
+      <c r="I54" s="133" t="s">
         <v>372</v>
       </c>
-      <c r="J54" s="137"/>
-      <c r="K54" s="137"/>
+      <c r="J54" s="133"/>
+      <c r="K54" s="133"/>
       <c r="L54" s="16">
         <f>MAX(L$3:L$51)</f>
         <v>0.25</v>
@@ -41809,37 +41809,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.75">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="126" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="135" t="s">
         <v>177</v>
       </c>
       <c r="D1" s="142"/>
       <c r="E1" s="142"/>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="136" t="s">
         <v>377</v>
       </c>
       <c r="G1" s="143"/>
       <c r="H1" s="143"/>
-      <c r="I1" s="128" t="s">
+      <c r="I1" s="137" t="s">
         <v>525</v>
       </c>
       <c r="J1" s="144"/>
       <c r="K1" s="144"/>
-      <c r="L1" s="132" t="s">
+      <c r="L1" s="128" t="s">
         <v>210</v>
       </c>
-      <c r="M1" s="133"/>
+      <c r="M1" s="129"/>
       <c r="N1" s="138"/>
       <c r="O1" s="138"/>
     </row>
     <row r="2" spans="1:15" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
@@ -44381,7 +44381,7 @@
       </c>
     </row>
     <row r="52" spans="1:15" ht="18.75">
-      <c r="I52" s="135" t="s">
+      <c r="I52" s="131" t="s">
         <v>370</v>
       </c>
       <c r="J52" s="139"/>
@@ -44404,7 +44404,7 @@
       </c>
     </row>
     <row r="53" spans="1:15" ht="18.75">
-      <c r="I53" s="136" t="s">
+      <c r="I53" s="132" t="s">
         <v>371</v>
       </c>
       <c r="J53" s="140"/>
@@ -44427,7 +44427,7 @@
       </c>
     </row>
     <row r="54" spans="1:15" ht="18.75">
-      <c r="I54" s="137" t="s">
+      <c r="I54" s="133" t="s">
         <v>372</v>
       </c>
       <c r="J54" s="141"/>
@@ -44636,37 +44636,37 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="15.75" customHeight="1">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="126" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="135" t="s">
         <v>177</v>
       </c>
       <c r="D1" s="142"/>
       <c r="E1" s="142"/>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="136" t="s">
         <v>377</v>
       </c>
       <c r="G1" s="143"/>
       <c r="H1" s="143"/>
-      <c r="I1" s="128" t="s">
+      <c r="I1" s="137" t="s">
         <v>525</v>
       </c>
       <c r="J1" s="144"/>
       <c r="K1" s="144"/>
-      <c r="L1" s="132" t="s">
+      <c r="L1" s="128" t="s">
         <v>210</v>
       </c>
-      <c r="M1" s="133"/>
+      <c r="M1" s="129"/>
       <c r="N1" s="138"/>
       <c r="O1" s="138"/>
     </row>
     <row r="2" spans="1:15" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
@@ -47208,7 +47208,7 @@
       </c>
     </row>
     <row r="52" spans="1:15" ht="18.75">
-      <c r="I52" s="135" t="s">
+      <c r="I52" s="131" t="s">
         <v>370</v>
       </c>
       <c r="J52" s="139"/>
@@ -47231,7 +47231,7 @@
       </c>
     </row>
     <row r="53" spans="1:15" ht="18.75">
-      <c r="I53" s="136" t="s">
+      <c r="I53" s="132" t="s">
         <v>371</v>
       </c>
       <c r="J53" s="140"/>
@@ -47254,7 +47254,7 @@
       </c>
     </row>
     <row r="54" spans="1:15" ht="18.75">
-      <c r="I54" s="137" t="s">
+      <c r="I54" s="133" t="s">
         <v>372</v>
       </c>
       <c r="J54" s="141"/>
@@ -47466,44 +47466,44 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="15.75" customHeight="1">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="126" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="135" t="s">
         <v>177</v>
       </c>
       <c r="D1" s="142"/>
       <c r="E1" s="142"/>
-      <c r="F1" s="127" t="s">
+      <c r="F1" s="136" t="s">
         <v>377</v>
       </c>
       <c r="G1" s="143"/>
       <c r="H1" s="143"/>
-      <c r="I1" s="128" t="s">
+      <c r="I1" s="137" t="s">
         <v>525</v>
       </c>
       <c r="J1" s="144"/>
       <c r="K1" s="144"/>
-      <c r="L1" s="129" t="s">
+      <c r="L1" s="125" t="s">
         <v>575</v>
       </c>
       <c r="M1" s="145"/>
       <c r="N1" s="146"/>
-      <c r="O1" s="132" t="s">
+      <c r="O1" s="128" t="s">
         <v>210</v>
       </c>
-      <c r="P1" s="133"/>
-      <c r="Q1" s="133"/>
+      <c r="P1" s="129"/>
+      <c r="Q1" s="129"/>
       <c r="R1" s="138"/>
       <c r="S1" s="138"/>
       <c r="T1" s="147"/>
     </row>
     <row r="2" spans="1:20" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
@@ -50844,7 +50844,7 @@
       </c>
     </row>
     <row r="52" spans="1:20" ht="18.75">
-      <c r="I52" s="135" t="s">
+      <c r="I52" s="131" t="s">
         <v>370</v>
       </c>
       <c r="J52" s="139"/>
@@ -50878,7 +50878,7 @@
       </c>
     </row>
     <row r="53" spans="1:20" ht="18.75">
-      <c r="I53" s="136" t="s">
+      <c r="I53" s="132" t="s">
         <v>371</v>
       </c>
       <c r="J53" s="140"/>
@@ -50912,7 +50912,7 @@
       </c>
     </row>
     <row r="54" spans="1:20" ht="18.75">
-      <c r="I54" s="137" t="s">
+      <c r="I54" s="133" t="s">
         <v>372</v>
       </c>
       <c r="J54" s="141"/>
@@ -50967,16 +50967,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="O1:T1"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="I54:K54"/>
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="B1:B2"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="O1:T1"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="I54:K54"/>
   </mergeCells>
   <conditionalFormatting sqref="O1:O2">
     <cfRule type="colorScale" priority="11">
@@ -51169,46 +51169,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:22" ht="15.75">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="126" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="135" t="s">
         <v>178</v>
       </c>
-      <c r="D1" s="126"/>
-      <c r="E1" s="126"/>
-      <c r="F1" s="127" t="s">
+      <c r="D1" s="135"/>
+      <c r="E1" s="135"/>
+      <c r="F1" s="136" t="s">
         <v>377</v>
       </c>
-      <c r="G1" s="127"/>
-      <c r="H1" s="127"/>
-      <c r="I1" s="128" t="s">
+      <c r="G1" s="136"/>
+      <c r="H1" s="136"/>
+      <c r="I1" s="137" t="s">
         <v>525</v>
       </c>
-      <c r="J1" s="128"/>
-      <c r="K1" s="128"/>
-      <c r="L1" s="129" t="s">
+      <c r="J1" s="137"/>
+      <c r="K1" s="137"/>
+      <c r="L1" s="125" t="s">
         <v>575</v>
       </c>
-      <c r="M1" s="130"/>
-      <c r="N1" s="131"/>
-      <c r="O1" s="148" t="s">
+      <c r="M1" s="126"/>
+      <c r="N1" s="127"/>
+      <c r="O1" s="159" t="s">
         <v>210</v>
       </c>
-      <c r="P1" s="149"/>
-      <c r="Q1" s="149"/>
-      <c r="R1" s="149"/>
-      <c r="S1" s="149"/>
-      <c r="T1" s="149"/>
-      <c r="U1" s="149"/>
-      <c r="V1" s="149"/>
+      <c r="P1" s="160"/>
+      <c r="Q1" s="160"/>
+      <c r="R1" s="160"/>
+      <c r="S1" s="160"/>
+      <c r="T1" s="160"/>
+      <c r="U1" s="160"/>
+      <c r="V1" s="160"/>
     </row>
     <row r="2" spans="1:22" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="32" t="s">
         <v>1</v>
       </c>
@@ -53866,17 +53866,17 @@
         <v>-3.83</v>
       </c>
       <c r="X36" s="102"/>
-      <c r="Y36" s="153" t="s">
+      <c r="Y36" s="151" t="s">
         <v>688</v>
       </c>
-      <c r="Z36" s="153"/>
-      <c r="AA36" s="153"/>
-      <c r="AB36" s="153"/>
-      <c r="AC36" s="153"/>
-      <c r="AD36" s="153"/>
-      <c r="AE36" s="153"/>
-      <c r="AF36" s="153"/>
-      <c r="AG36" s="153"/>
+      <c r="Z36" s="151"/>
+      <c r="AA36" s="151"/>
+      <c r="AB36" s="151"/>
+      <c r="AC36" s="151"/>
+      <c r="AD36" s="151"/>
+      <c r="AE36" s="151"/>
+      <c r="AF36" s="151"/>
+      <c r="AG36" s="151"/>
       <c r="AH36" s="102"/>
       <c r="AI36" s="102"/>
     </row>
@@ -53956,23 +53956,23 @@
         <v>-1.63</v>
       </c>
       <c r="X37" s="101"/>
-      <c r="Y37" s="160" t="s">
+      <c r="Y37" s="158" t="s">
         <v>687</v>
       </c>
-      <c r="Z37" s="160"/>
-      <c r="AA37" s="157" t="s">
+      <c r="Z37" s="158"/>
+      <c r="AA37" s="155" t="s">
         <v>686</v>
       </c>
-      <c r="AB37" s="157"/>
-      <c r="AC37" s="158" t="s">
+      <c r="AB37" s="155"/>
+      <c r="AC37" s="156" t="s">
         <v>685</v>
       </c>
-      <c r="AD37" s="158"/>
-      <c r="AE37" s="159" t="s">
+      <c r="AD37" s="156"/>
+      <c r="AE37" s="157" t="s">
         <v>684</v>
       </c>
-      <c r="AF37" s="159"/>
-      <c r="AG37" s="159"/>
+      <c r="AF37" s="157"/>
+      <c r="AG37" s="157"/>
       <c r="AH37" s="103"/>
       <c r="AI37" s="103"/>
     </row>
@@ -54052,27 +54052,27 @@
         <v>30.33</v>
       </c>
       <c r="X38" s="91"/>
-      <c r="Y38" s="150">
+      <c r="Y38" s="148">
         <f>E3</f>
         <v>1083.5999999999999</v>
       </c>
-      <c r="Z38" s="151"/>
-      <c r="AA38" s="154">
+      <c r="Z38" s="149"/>
+      <c r="AA38" s="152">
         <f>H3</f>
         <v>413.19</v>
       </c>
-      <c r="AB38" s="155"/>
-      <c r="AC38" s="154">
+      <c r="AB38" s="153"/>
+      <c r="AC38" s="152">
         <f>K3</f>
         <v>88.44</v>
       </c>
-      <c r="AD38" s="155"/>
-      <c r="AE38" s="154">
+      <c r="AD38" s="153"/>
+      <c r="AE38" s="152">
         <f>N3</f>
         <v>22.07</v>
       </c>
-      <c r="AF38" s="155"/>
-      <c r="AG38" s="155"/>
+      <c r="AF38" s="153"/>
+      <c r="AG38" s="153"/>
       <c r="AH38" s="104"/>
       <c r="AI38" s="104"/>
     </row>
@@ -54152,26 +54152,26 @@
         <v>7.07</v>
       </c>
       <c r="X39" s="100"/>
-      <c r="Y39" s="152" t="s">
+      <c r="Y39" s="150" t="s">
         <v>689</v>
       </c>
-      <c r="Z39" s="152"/>
-      <c r="AA39" s="156">
+      <c r="Z39" s="150"/>
+      <c r="AA39" s="154">
         <f>$Y$38/AA38</f>
         <v>2.6225223262905684</v>
       </c>
-      <c r="AB39" s="156"/>
-      <c r="AC39" s="156">
+      <c r="AB39" s="154"/>
+      <c r="AC39" s="154">
         <f>$Y$38/AC38</f>
         <v>12.252374491180461</v>
       </c>
-      <c r="AD39" s="156"/>
-      <c r="AE39" s="156">
+      <c r="AD39" s="154"/>
+      <c r="AE39" s="154">
         <f>$Y$38/AE38</f>
         <v>49.098323516085181</v>
       </c>
-      <c r="AF39" s="156"/>
-      <c r="AG39" s="156"/>
+      <c r="AF39" s="154"/>
+      <c r="AG39" s="154"/>
       <c r="AH39" s="100"/>
       <c r="AI39" s="100"/>
     </row>
@@ -55196,11 +55196,11 @@
       </c>
     </row>
     <row r="52" spans="1:22" ht="30.75" customHeight="1">
-      <c r="I52" s="135" t="s">
+      <c r="I52" s="131" t="s">
         <v>370</v>
       </c>
-      <c r="J52" s="135"/>
-      <c r="K52" s="135"/>
+      <c r="J52" s="131"/>
+      <c r="K52" s="131"/>
       <c r="L52" s="37"/>
       <c r="M52" s="52"/>
       <c r="N52" s="52"/>
@@ -55238,11 +55238,11 @@
       </c>
     </row>
     <row r="53" spans="1:22" ht="30.75" customHeight="1">
-      <c r="I53" s="136" t="s">
+      <c r="I53" s="132" t="s">
         <v>371</v>
       </c>
-      <c r="J53" s="136"/>
-      <c r="K53" s="136"/>
+      <c r="J53" s="132"/>
+      <c r="K53" s="132"/>
       <c r="L53" s="38"/>
       <c r="M53" s="53"/>
       <c r="N53" s="53"/>
@@ -55280,11 +55280,11 @@
       </c>
     </row>
     <row r="54" spans="1:22" ht="30.75" customHeight="1">
-      <c r="I54" s="137" t="s">
+      <c r="I54" s="133" t="s">
         <v>372</v>
       </c>
-      <c r="J54" s="137"/>
-      <c r="K54" s="137"/>
+      <c r="J54" s="133"/>
+      <c r="K54" s="133"/>
       <c r="L54" s="39"/>
       <c r="M54" s="54"/>
       <c r="N54" s="54"/>
@@ -55349,6 +55349,16 @@
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="L1:N1"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="I54:K54"/>
+    <mergeCell ref="O1:V1"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:E1"/>
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="Y38:Z38"/>
     <mergeCell ref="Y39:Z39"/>
     <mergeCell ref="Y36:AG36"/>
@@ -55362,16 +55372,6 @@
     <mergeCell ref="AC37:AD37"/>
     <mergeCell ref="AE37:AG37"/>
     <mergeCell ref="Y37:Z37"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:E1"/>
-    <mergeCell ref="F1:H1"/>
-    <mergeCell ref="I1:K1"/>
-    <mergeCell ref="L1:N1"/>
-    <mergeCell ref="I52:K52"/>
-    <mergeCell ref="I53:K53"/>
-    <mergeCell ref="I54:K54"/>
-    <mergeCell ref="O1:V1"/>
   </mergeCells>
   <conditionalFormatting sqref="O1:O2">
     <cfRule type="colorScale" priority="18">
@@ -55638,35 +55638,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="15.75">
-      <c r="A1" s="125" t="s">
+      <c r="A1" s="134" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="125" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="127" t="s">
+      <c r="B1" s="134" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="136" t="s">
         <v>377</v>
       </c>
-      <c r="D1" s="127"/>
-      <c r="E1" s="127"/>
-      <c r="F1" s="128" t="s">
+      <c r="D1" s="136"/>
+      <c r="E1" s="136"/>
+      <c r="F1" s="137" t="s">
         <v>525</v>
       </c>
-      <c r="G1" s="128"/>
-      <c r="H1" s="128"/>
-      <c r="I1" s="129" t="s">
+      <c r="G1" s="137"/>
+      <c r="H1" s="137"/>
+      <c r="I1" s="125" t="s">
         <v>575</v>
       </c>
-      <c r="J1" s="130"/>
-      <c r="K1" s="131"/>
-      <c r="L1" s="133" t="s">
+      <c r="J1" s="126"/>
+      <c r="K1" s="127"/>
+      <c r="L1" s="129" t="s">
         <v>210</v>
       </c>
-      <c r="M1" s="134"/>
+      <c r="M1" s="130"/>
     </row>
     <row r="2" spans="1:13" ht="31.5">
-      <c r="A2" s="125"/>
-      <c r="B2" s="125"/>
+      <c r="A2" s="134"/>
+      <c r="B2" s="134"/>
       <c r="C2" s="40" t="s">
         <v>1</v>
       </c>
@@ -57809,11 +57809,11 @@
       </c>
     </row>
     <row r="52" spans="1:13" ht="30.75" customHeight="1">
-      <c r="F52" s="135" t="s">
+      <c r="F52" s="131" t="s">
         <v>370</v>
       </c>
-      <c r="G52" s="135"/>
-      <c r="H52" s="135"/>
+      <c r="G52" s="131"/>
+      <c r="H52" s="131"/>
       <c r="I52" s="37"/>
       <c r="J52" s="52"/>
       <c r="K52" s="52"/>
@@ -57827,11 +57827,11 @@
       </c>
     </row>
     <row r="53" spans="1:13" ht="30.75" customHeight="1">
-      <c r="F53" s="136" t="s">
+      <c r="F53" s="132" t="s">
         <v>371</v>
       </c>
-      <c r="G53" s="136"/>
-      <c r="H53" s="136"/>
+      <c r="G53" s="132"/>
+      <c r="H53" s="132"/>
       <c r="I53" s="38"/>
       <c r="J53" s="53"/>
       <c r="K53" s="53"/>
@@ -57845,11 +57845,11 @@
       </c>
     </row>
     <row r="54" spans="1:13" ht="30.75" customHeight="1">
-      <c r="F54" s="137" t="s">
+      <c r="F54" s="133" t="s">
         <v>372</v>
       </c>
-      <c r="G54" s="137"/>
-      <c r="H54" s="137"/>
+      <c r="G54" s="133"/>
+      <c r="H54" s="133"/>
       <c r="I54" s="39"/>
       <c r="J54" s="54"/>
       <c r="K54" s="54"/>
@@ -57962,46 +57962,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18.75">
-      <c r="A1" s="168" t="s">
+      <c r="A1" s="163" t="s">
         <v>692</v>
       </c>
-      <c r="B1" s="168"/>
-      <c r="C1" s="168"/>
-      <c r="D1" s="168"/>
-      <c r="E1" s="168"/>
+      <c r="B1" s="163"/>
+      <c r="C1" s="163"/>
+      <c r="D1" s="163"/>
+      <c r="E1" s="163"/>
       <c r="G1" s="76"/>
       <c r="H1" s="91"/>
-      <c r="I1" s="165"/>
-      <c r="J1" s="165"/>
-      <c r="K1" s="165"/>
-      <c r="L1" s="165"/>
-      <c r="M1" s="165"/>
-      <c r="N1" s="165"/>
-      <c r="O1" s="165"/>
-      <c r="P1" s="165"/>
-      <c r="Q1" s="165"/>
+      <c r="I1" s="164"/>
+      <c r="J1" s="164"/>
+      <c r="K1" s="164"/>
+      <c r="L1" s="164"/>
+      <c r="M1" s="164"/>
+      <c r="N1" s="164"/>
+      <c r="O1" s="164"/>
+      <c r="P1" s="164"/>
+      <c r="Q1" s="164"/>
     </row>
     <row r="2" spans="1:18" ht="18.75">
-      <c r="A2" s="168"/>
-      <c r="B2" s="168"/>
-      <c r="C2" s="168"/>
-      <c r="D2" s="168"/>
-      <c r="E2" s="168"/>
+      <c r="A2" s="163"/>
+      <c r="B2" s="163"/>
+      <c r="C2" s="163"/>
+      <c r="D2" s="163"/>
+      <c r="E2" s="163"/>
       <c r="G2" s="76"/>
       <c r="H2" s="113" t="s">
         <v>757</v>
       </c>
-      <c r="I2" s="166" t="s">
+      <c r="I2" s="165" t="s">
         <v>762</v>
       </c>
-      <c r="J2" s="166"/>
-      <c r="K2" s="166"/>
-      <c r="L2" s="166"/>
-      <c r="M2" s="166"/>
-      <c r="N2" s="166"/>
-      <c r="O2" s="166"/>
-      <c r="P2" s="166"/>
-      <c r="Q2" s="166"/>
+      <c r="J2" s="165"/>
+      <c r="K2" s="165"/>
+      <c r="L2" s="165"/>
+      <c r="M2" s="165"/>
+      <c r="N2" s="165"/>
+      <c r="O2" s="165"/>
+      <c r="P2" s="165"/>
+      <c r="Q2" s="165"/>
     </row>
     <row r="3" spans="1:18" ht="18.75">
       <c r="A3" s="107" t="s">
@@ -58023,17 +58023,17 @@
       <c r="H3" s="113" t="s">
         <v>758</v>
       </c>
-      <c r="I3" s="166" t="s">
+      <c r="I3" s="165" t="s">
         <v>763</v>
       </c>
-      <c r="J3" s="166"/>
-      <c r="K3" s="166"/>
-      <c r="L3" s="166"/>
-      <c r="M3" s="166"/>
-      <c r="N3" s="166"/>
-      <c r="O3" s="166"/>
-      <c r="P3" s="166"/>
-      <c r="Q3" s="166"/>
+      <c r="J3" s="165"/>
+      <c r="K3" s="165"/>
+      <c r="L3" s="165"/>
+      <c r="M3" s="165"/>
+      <c r="N3" s="165"/>
+      <c r="O3" s="165"/>
+      <c r="P3" s="165"/>
+      <c r="Q3" s="165"/>
     </row>
     <row r="4" spans="1:18" ht="45">
       <c r="A4" s="108" t="s">
@@ -58051,20 +58051,20 @@
       <c r="E4" s="70">
         <v>38.06</v>
       </c>
-      <c r="F4" s="162" t="s">
+      <c r="F4" s="166" t="s">
         <v>757</v>
       </c>
       <c r="G4" s="112"/>
       <c r="H4" s="91"/>
-      <c r="I4" s="165"/>
-      <c r="J4" s="165"/>
-      <c r="K4" s="165"/>
-      <c r="L4" s="165"/>
-      <c r="M4" s="165"/>
-      <c r="N4" s="165"/>
-      <c r="O4" s="165"/>
-      <c r="P4" s="165"/>
-      <c r="Q4" s="165"/>
+      <c r="I4" s="164"/>
+      <c r="J4" s="164"/>
+      <c r="K4" s="164"/>
+      <c r="L4" s="164"/>
+      <c r="M4" s="164"/>
+      <c r="N4" s="164"/>
+      <c r="O4" s="164"/>
+      <c r="P4" s="164"/>
+      <c r="Q4" s="164"/>
     </row>
     <row r="5" spans="1:18" ht="45">
       <c r="A5" s="108" t="s">
@@ -58082,18 +58082,18 @@
       <c r="E5" s="70">
         <v>21.1</v>
       </c>
-      <c r="F5" s="163"/>
+      <c r="F5" s="167"/>
       <c r="G5" s="112"/>
       <c r="H5" s="91"/>
-      <c r="I5" s="165"/>
-      <c r="J5" s="165"/>
-      <c r="K5" s="165"/>
-      <c r="L5" s="165"/>
-      <c r="M5" s="165"/>
-      <c r="N5" s="165"/>
-      <c r="O5" s="165"/>
-      <c r="P5" s="165"/>
-      <c r="Q5" s="165"/>
+      <c r="I5" s="164"/>
+      <c r="J5" s="164"/>
+      <c r="K5" s="164"/>
+      <c r="L5" s="164"/>
+      <c r="M5" s="164"/>
+      <c r="N5" s="164"/>
+      <c r="O5" s="164"/>
+      <c r="P5" s="164"/>
+      <c r="Q5" s="164"/>
     </row>
     <row r="6" spans="1:18" ht="45">
       <c r="A6" s="108" t="s">
@@ -58111,21 +58111,21 @@
       <c r="E6" s="70">
         <v>18.7</v>
       </c>
-      <c r="F6" s="163"/>
+      <c r="F6" s="167"/>
       <c r="G6" s="112"/>
-      <c r="H6" s="167" t="s">
+      <c r="H6" s="162" t="s">
         <v>761</v>
       </c>
-      <c r="I6" s="167"/>
-      <c r="J6" s="167"/>
-      <c r="K6" s="167"/>
-      <c r="L6" s="167"/>
-      <c r="M6" s="167"/>
-      <c r="N6" s="167"/>
-      <c r="O6" s="167"/>
-      <c r="P6" s="167"/>
-      <c r="Q6" s="167"/>
-      <c r="R6" s="167"/>
+      <c r="I6" s="162"/>
+      <c r="J6" s="162"/>
+      <c r="K6" s="162"/>
+      <c r="L6" s="162"/>
+      <c r="M6" s="162"/>
+      <c r="N6" s="162"/>
+      <c r="O6" s="162"/>
+      <c r="P6" s="162"/>
+      <c r="Q6" s="162"/>
+      <c r="R6" s="162"/>
     </row>
     <row r="7" spans="1:18" ht="45">
       <c r="A7" s="108" t="s">
@@ -58143,29 +58143,29 @@
       <c r="E7" s="70">
         <v>8.99</v>
       </c>
-      <c r="F7" s="163"/>
+      <c r="F7" s="167"/>
       <c r="G7" s="112"/>
       <c r="H7" s="122"/>
-      <c r="I7" s="164">
+      <c r="I7" s="161">
         <v>20</v>
       </c>
-      <c r="J7" s="164"/>
-      <c r="K7" s="164">
+      <c r="J7" s="161"/>
+      <c r="K7" s="161">
         <v>21</v>
       </c>
-      <c r="L7" s="164"/>
-      <c r="M7" s="164">
+      <c r="L7" s="161"/>
+      <c r="M7" s="161">
         <v>22</v>
       </c>
-      <c r="N7" s="164"/>
-      <c r="O7" s="164">
+      <c r="N7" s="161"/>
+      <c r="O7" s="161">
         <v>23</v>
       </c>
-      <c r="P7" s="164"/>
-      <c r="Q7" s="164">
+      <c r="P7" s="161"/>
+      <c r="Q7" s="161">
         <v>24</v>
       </c>
-      <c r="R7" s="164"/>
+      <c r="R7" s="161"/>
     </row>
     <row r="8" spans="1:18" ht="45">
       <c r="A8" s="108" t="s">
@@ -58183,7 +58183,7 @@
       <c r="E8" s="70">
         <v>0.96</v>
       </c>
-      <c r="F8" s="163"/>
+      <c r="F8" s="167"/>
       <c r="G8" s="112"/>
       <c r="H8" s="105" t="s">
         <v>756</v>
@@ -58235,7 +58235,7 @@
       <c r="E9" s="70">
         <v>1</v>
       </c>
-      <c r="F9" s="163"/>
+      <c r="F9" s="167"/>
       <c r="G9" s="112"/>
       <c r="H9" s="105">
         <v>1</v>
@@ -58283,7 +58283,7 @@
       <c r="E10" s="70">
         <v>1.3</v>
       </c>
-      <c r="F10" s="163"/>
+      <c r="F10" s="167"/>
       <c r="G10" s="112"/>
       <c r="H10" s="105">
         <v>2</v>
@@ -58331,7 +58331,7 @@
       <c r="E11" s="116">
         <v>69.87</v>
       </c>
-      <c r="F11" s="162" t="s">
+      <c r="F11" s="166" t="s">
         <v>758</v>
       </c>
       <c r="H11" s="105">
@@ -58380,7 +58380,7 @@
       <c r="E12" s="116">
         <v>36.119999999999997</v>
       </c>
-      <c r="F12" s="163"/>
+      <c r="F12" s="167"/>
       <c r="H12" s="105">
         <v>4</v>
       </c>
@@ -58427,7 +58427,7 @@
       <c r="E13" s="116">
         <v>38.89</v>
       </c>
-      <c r="F13" s="163"/>
+      <c r="F13" s="167"/>
       <c r="H13" s="98">
         <v>5</v>
       </c>
@@ -58488,7 +58488,7 @@
       <c r="E14" s="116">
         <v>20.6</v>
       </c>
-      <c r="F14" s="163"/>
+      <c r="F14" s="167"/>
     </row>
     <row r="15" spans="1:18" ht="45">
       <c r="A15" s="120" t="s">
@@ -58506,21 +58506,21 @@
       <c r="E15" s="116">
         <v>5.87</v>
       </c>
-      <c r="F15" s="163"/>
+      <c r="F15" s="167"/>
       <c r="H15" s="123">
         <v>1</v>
       </c>
-      <c r="I15" s="161" t="s">
+      <c r="I15" s="168" t="s">
         <v>678</v>
       </c>
-      <c r="J15" s="161"/>
-      <c r="K15" s="161"/>
-      <c r="L15" s="161"/>
-      <c r="M15" s="161"/>
-      <c r="N15" s="161"/>
-      <c r="O15" s="161"/>
-      <c r="P15" s="161"/>
-      <c r="Q15" s="161"/>
+      <c r="J15" s="168"/>
+      <c r="K15" s="168"/>
+      <c r="L15" s="168"/>
+      <c r="M15" s="168"/>
+      <c r="N15" s="168"/>
+      <c r="O15" s="168"/>
+      <c r="P15" s="168"/>
+      <c r="Q15" s="168"/>
     </row>
     <row r="16" spans="1:18" ht="45">
       <c r="A16" s="120" t="s">
@@ -58538,21 +58538,21 @@
       <c r="E16" s="116">
         <v>6.09</v>
       </c>
-      <c r="F16" s="163"/>
+      <c r="F16" s="167"/>
       <c r="H16" s="123">
         <v>2</v>
       </c>
-      <c r="I16" s="161" t="s">
+      <c r="I16" s="168" t="s">
         <v>677</v>
       </c>
-      <c r="J16" s="161"/>
-      <c r="K16" s="161"/>
-      <c r="L16" s="161"/>
-      <c r="M16" s="161"/>
-      <c r="N16" s="161"/>
-      <c r="O16" s="161"/>
-      <c r="P16" s="161"/>
-      <c r="Q16" s="161"/>
+      <c r="J16" s="168"/>
+      <c r="K16" s="168"/>
+      <c r="L16" s="168"/>
+      <c r="M16" s="168"/>
+      <c r="N16" s="168"/>
+      <c r="O16" s="168"/>
+      <c r="P16" s="168"/>
+      <c r="Q16" s="168"/>
     </row>
     <row r="17" spans="1:17" ht="45">
       <c r="A17" s="120" t="s">
@@ -58570,56 +58570,65 @@
       <c r="E17" s="116">
         <v>6.42</v>
       </c>
-      <c r="F17" s="163"/>
+      <c r="F17" s="167"/>
       <c r="H17" s="123">
         <v>3</v>
       </c>
-      <c r="I17" s="161" t="s">
+      <c r="I17" s="168" t="s">
         <v>679</v>
       </c>
-      <c r="J17" s="161"/>
-      <c r="K17" s="161"/>
-      <c r="L17" s="161"/>
-      <c r="M17" s="161"/>
-      <c r="N17" s="161"/>
-      <c r="O17" s="161"/>
-      <c r="P17" s="161"/>
-      <c r="Q17" s="161"/>
+      <c r="J17" s="168"/>
+      <c r="K17" s="168"/>
+      <c r="L17" s="168"/>
+      <c r="M17" s="168"/>
+      <c r="N17" s="168"/>
+      <c r="O17" s="168"/>
+      <c r="P17" s="168"/>
+      <c r="Q17" s="168"/>
     </row>
     <row r="18" spans="1:17" ht="18.75">
       <c r="H18" s="123">
         <v>4</v>
       </c>
-      <c r="I18" s="161" t="s">
+      <c r="I18" s="168" t="s">
         <v>680</v>
       </c>
-      <c r="J18" s="161"/>
-      <c r="K18" s="161"/>
-      <c r="L18" s="161"/>
-      <c r="M18" s="161"/>
-      <c r="N18" s="161"/>
-      <c r="O18" s="161"/>
-      <c r="P18" s="161"/>
-      <c r="Q18" s="161"/>
+      <c r="J18" s="168"/>
+      <c r="K18" s="168"/>
+      <c r="L18" s="168"/>
+      <c r="M18" s="168"/>
+      <c r="N18" s="168"/>
+      <c r="O18" s="168"/>
+      <c r="P18" s="168"/>
+      <c r="Q18" s="168"/>
     </row>
     <row r="19" spans="1:17" ht="18.75">
       <c r="H19" s="123">
         <v>5</v>
       </c>
-      <c r="I19" s="161" t="s">
+      <c r="I19" s="168" t="s">
         <v>681</v>
       </c>
-      <c r="J19" s="161"/>
-      <c r="K19" s="161"/>
-      <c r="L19" s="161"/>
-      <c r="M19" s="161"/>
-      <c r="N19" s="161"/>
-      <c r="O19" s="161"/>
-      <c r="P19" s="161"/>
-      <c r="Q19" s="161"/>
+      <c r="J19" s="168"/>
+      <c r="K19" s="168"/>
+      <c r="L19" s="168"/>
+      <c r="M19" s="168"/>
+      <c r="N19" s="168"/>
+      <c r="O19" s="168"/>
+      <c r="P19" s="168"/>
+      <c r="Q19" s="168"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="I18:Q18"/>
+    <mergeCell ref="I19:Q19"/>
+    <mergeCell ref="F11:F17"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:P7"/>
+    <mergeCell ref="I15:Q15"/>
+    <mergeCell ref="I16:Q16"/>
+    <mergeCell ref="I17:Q17"/>
     <mergeCell ref="Q7:R7"/>
     <mergeCell ref="H6:R6"/>
     <mergeCell ref="I7:J7"/>
@@ -58630,15 +58639,6 @@
     <mergeCell ref="I4:Q4"/>
     <mergeCell ref="I5:Q5"/>
     <mergeCell ref="F4:F10"/>
-    <mergeCell ref="F11:F17"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:P7"/>
-    <mergeCell ref="I15:Q15"/>
-    <mergeCell ref="I16:Q16"/>
-    <mergeCell ref="I17:Q17"/>
-    <mergeCell ref="I18:Q18"/>
-    <mergeCell ref="I19:Q19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -58661,62 +58661,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:34" s="1" customFormat="1" ht="21.75" thickBot="1">
-      <c r="A1" s="172" t="s">
+      <c r="A1" s="176" t="s">
         <v>682</v>
       </c>
-      <c r="B1" s="172"/>
-      <c r="C1" s="172"/>
-      <c r="D1" s="172"/>
-      <c r="E1" s="172"/>
-      <c r="F1" s="172"/>
-      <c r="G1" s="172"/>
-      <c r="H1" s="172"/>
-      <c r="I1" s="172"/>
-      <c r="J1" s="172"/>
-      <c r="L1" s="169" t="s">
+      <c r="B1" s="176"/>
+      <c r="C1" s="176"/>
+      <c r="D1" s="176"/>
+      <c r="E1" s="176"/>
+      <c r="F1" s="176"/>
+      <c r="G1" s="176"/>
+      <c r="H1" s="176"/>
+      <c r="I1" s="176"/>
+      <c r="J1" s="176"/>
+      <c r="L1" s="173" t="s">
         <v>629</v>
       </c>
-      <c r="M1" s="170"/>
-      <c r="N1" s="170"/>
-      <c r="O1" s="170"/>
-      <c r="P1" s="170"/>
-      <c r="Q1" s="170"/>
-      <c r="R1" s="170"/>
-      <c r="S1" s="170"/>
-      <c r="T1" s="170"/>
-      <c r="U1" s="170"/>
-      <c r="V1" s="171"/>
-      <c r="X1" s="169" t="s">
+      <c r="M1" s="174"/>
+      <c r="N1" s="174"/>
+      <c r="O1" s="174"/>
+      <c r="P1" s="174"/>
+      <c r="Q1" s="174"/>
+      <c r="R1" s="174"/>
+      <c r="S1" s="174"/>
+      <c r="T1" s="174"/>
+      <c r="U1" s="174"/>
+      <c r="V1" s="175"/>
+      <c r="X1" s="173" t="s">
         <v>631</v>
       </c>
-      <c r="Y1" s="170"/>
-      <c r="Z1" s="170"/>
-      <c r="AA1" s="170"/>
-      <c r="AB1" s="170"/>
-      <c r="AC1" s="170"/>
-      <c r="AD1" s="170"/>
-      <c r="AE1" s="170"/>
-      <c r="AF1" s="170"/>
-      <c r="AG1" s="170"/>
-      <c r="AH1" s="171"/>
+      <c r="Y1" s="174"/>
+      <c r="Z1" s="174"/>
+      <c r="AA1" s="174"/>
+      <c r="AB1" s="174"/>
+      <c r="AC1" s="174"/>
+      <c r="AD1" s="174"/>
+      <c r="AE1" s="174"/>
+      <c r="AF1" s="174"/>
+      <c r="AG1" s="174"/>
+      <c r="AH1" s="175"/>
     </row>
     <row r="2" spans="1:34" ht="36.75" customHeight="1">
       <c r="A2" s="61"/>
-      <c r="B2" s="127" t="s">
+      <c r="B2" s="136" t="s">
         <v>614</v>
       </c>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="128" t="s">
+      <c r="C2" s="136"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="137" t="s">
         <v>617</v>
       </c>
-      <c r="F2" s="128"/>
-      <c r="G2" s="128"/>
-      <c r="H2" s="173" t="s">
+      <c r="F2" s="137"/>
+      <c r="G2" s="137"/>
+      <c r="H2" s="177" t="s">
         <v>618</v>
       </c>
-      <c r="I2" s="173"/>
-      <c r="J2" s="173"/>
+      <c r="I2" s="177"/>
+      <c r="J2" s="177"/>
       <c r="L2" s="75"/>
       <c r="M2" s="76"/>
       <c r="N2" s="76"/>
@@ -59206,18 +59206,18 @@
       <c r="AH11" s="77"/>
     </row>
     <row r="12" spans="1:34" ht="21">
-      <c r="A12" s="172" t="s">
+      <c r="A12" s="176" t="s">
         <v>621</v>
       </c>
-      <c r="B12" s="172"/>
-      <c r="C12" s="172"/>
-      <c r="D12" s="172"/>
-      <c r="E12" s="172"/>
-      <c r="F12" s="172"/>
-      <c r="G12" s="172"/>
-      <c r="H12" s="172"/>
-      <c r="I12" s="172"/>
-      <c r="J12" s="172"/>
+      <c r="B12" s="176"/>
+      <c r="C12" s="176"/>
+      <c r="D12" s="176"/>
+      <c r="E12" s="176"/>
+      <c r="F12" s="176"/>
+      <c r="G12" s="176"/>
+      <c r="H12" s="176"/>
+      <c r="I12" s="176"/>
+      <c r="J12" s="176"/>
       <c r="L12" s="75"/>
       <c r="M12" s="76"/>
       <c r="N12" s="76"/>
@@ -59243,21 +59243,21 @@
     </row>
     <row r="13" spans="1:34" ht="35.25" customHeight="1">
       <c r="A13" s="61"/>
-      <c r="B13" s="127" t="s">
+      <c r="B13" s="136" t="s">
         <v>614</v>
       </c>
-      <c r="C13" s="127"/>
-      <c r="D13" s="127"/>
-      <c r="E13" s="128" t="s">
+      <c r="C13" s="136"/>
+      <c r="D13" s="136"/>
+      <c r="E13" s="137" t="s">
         <v>617</v>
       </c>
-      <c r="F13" s="128"/>
-      <c r="G13" s="128"/>
-      <c r="H13" s="173" t="s">
+      <c r="F13" s="137"/>
+      <c r="G13" s="137"/>
+      <c r="H13" s="177" t="s">
         <v>618</v>
       </c>
-      <c r="I13" s="173"/>
-      <c r="J13" s="173"/>
+      <c r="I13" s="177"/>
+      <c r="J13" s="177"/>
       <c r="L13" s="75"/>
       <c r="M13" s="76"/>
       <c r="N13" s="76"/>
@@ -59526,19 +59526,19 @@
         <f>'15 Elementos'!T54</f>
         <v>1.1399999999999999</v>
       </c>
-      <c r="L18" s="169" t="s">
+      <c r="L18" s="173" t="s">
         <v>630</v>
       </c>
-      <c r="M18" s="170"/>
-      <c r="N18" s="170"/>
-      <c r="O18" s="170"/>
-      <c r="P18" s="170"/>
-      <c r="Q18" s="170"/>
-      <c r="R18" s="170"/>
-      <c r="S18" s="170"/>
-      <c r="T18" s="170"/>
-      <c r="U18" s="170"/>
-      <c r="V18" s="171"/>
+      <c r="M18" s="174"/>
+      <c r="N18" s="174"/>
+      <c r="O18" s="174"/>
+      <c r="P18" s="174"/>
+      <c r="Q18" s="174"/>
+      <c r="R18" s="174"/>
+      <c r="S18" s="174"/>
+      <c r="T18" s="174"/>
+      <c r="U18" s="174"/>
+      <c r="V18" s="175"/>
       <c r="X18" s="75"/>
       <c r="Y18" s="76"/>
       <c r="Z18" s="76"/>
@@ -59886,19 +59886,19 @@
       <c r="A27" s="94" t="s">
         <v>676</v>
       </c>
-      <c r="B27" s="157" t="s">
+      <c r="B27" s="155" t="s">
         <v>686</v>
       </c>
-      <c r="C27" s="157"/>
-      <c r="D27" s="174" t="s">
+      <c r="C27" s="155"/>
+      <c r="D27" s="178" t="s">
         <v>685</v>
       </c>
-      <c r="E27" s="175"/>
-      <c r="F27" s="159" t="s">
+      <c r="E27" s="179"/>
+      <c r="F27" s="157" t="s">
         <v>684</v>
       </c>
-      <c r="G27" s="159"/>
-      <c r="H27" s="159"/>
+      <c r="G27" s="157"/>
+      <c r="H27" s="157"/>
       <c r="I27" s="95" t="s">
         <v>529</v>
       </c>
@@ -59932,19 +59932,19 @@
       <c r="A28" s="90">
         <v>1</v>
       </c>
-      <c r="B28" s="161">
+      <c r="B28" s="168">
         <v>0.35</v>
       </c>
-      <c r="C28" s="161"/>
-      <c r="D28" s="176">
+      <c r="C28" s="168"/>
+      <c r="D28" s="169">
         <v>0.33</v>
       </c>
-      <c r="E28" s="177"/>
-      <c r="F28" s="161">
+      <c r="E28" s="170"/>
+      <c r="F28" s="168">
         <v>0.27</v>
       </c>
-      <c r="G28" s="161"/>
-      <c r="H28" s="161"/>
+      <c r="G28" s="168"/>
+      <c r="H28" s="168"/>
       <c r="I28" s="99">
         <f>B28/D28</f>
         <v>1.0606060606060606</v>
@@ -59980,19 +59980,19 @@
       <c r="A29" s="90">
         <v>2</v>
       </c>
-      <c r="B29" s="161">
+      <c r="B29" s="168">
         <v>829.35</v>
       </c>
-      <c r="C29" s="161"/>
-      <c r="D29" s="176">
+      <c r="C29" s="168"/>
+      <c r="D29" s="169">
         <v>148.22</v>
       </c>
-      <c r="E29" s="177"/>
-      <c r="F29" s="161">
+      <c r="E29" s="170"/>
+      <c r="F29" s="168">
         <v>4.28</v>
       </c>
-      <c r="G29" s="161"/>
-      <c r="H29" s="161"/>
+      <c r="G29" s="168"/>
+      <c r="H29" s="168"/>
       <c r="I29" s="99">
         <f t="shared" ref="I29:I31" si="2">B29/D29</f>
         <v>5.595398731615167</v>
@@ -60028,19 +60028,19 @@
       <c r="A30" s="90">
         <v>3</v>
       </c>
-      <c r="B30" s="161">
+      <c r="B30" s="168">
         <v>14.05</v>
       </c>
-      <c r="C30" s="161"/>
-      <c r="D30" s="176">
+      <c r="C30" s="168"/>
+      <c r="D30" s="169">
         <v>20.03</v>
       </c>
-      <c r="E30" s="177"/>
-      <c r="F30" s="161">
+      <c r="E30" s="170"/>
+      <c r="F30" s="168">
         <v>13.32</v>
       </c>
-      <c r="G30" s="161"/>
-      <c r="H30" s="161"/>
+      <c r="G30" s="168"/>
+      <c r="H30" s="168"/>
       <c r="I30" s="99">
         <f t="shared" si="2"/>
         <v>0.70144782825761354</v>
@@ -60076,19 +60076,19 @@
       <c r="A31" s="90">
         <v>4</v>
       </c>
-      <c r="B31" s="161">
+      <c r="B31" s="168">
         <v>0.23</v>
       </c>
-      <c r="C31" s="161"/>
-      <c r="D31" s="161">
+      <c r="C31" s="168"/>
+      <c r="D31" s="168">
         <v>22.95</v>
       </c>
-      <c r="E31" s="161"/>
-      <c r="F31" s="161">
+      <c r="E31" s="168"/>
+      <c r="F31" s="168">
         <v>23.72</v>
       </c>
-      <c r="G31" s="161"/>
-      <c r="H31" s="161"/>
+      <c r="G31" s="168"/>
+      <c r="H31" s="168"/>
       <c r="I31" s="99">
         <f t="shared" si="2"/>
         <v>1.0021786492374729E-2</v>
@@ -60124,22 +60124,22 @@
       <c r="A32" s="93">
         <v>5</v>
       </c>
-      <c r="B32" s="179">
+      <c r="B32" s="172">
         <f>SUM(B28:C31)</f>
         <v>843.98</v>
       </c>
-      <c r="C32" s="179"/>
-      <c r="D32" s="179">
+      <c r="C32" s="172"/>
+      <c r="D32" s="172">
         <f>SUM(D28:E31)</f>
         <v>191.53</v>
       </c>
-      <c r="E32" s="179"/>
-      <c r="F32" s="179">
+      <c r="E32" s="172"/>
+      <c r="F32" s="172">
         <f>SUM(F28:H31)</f>
         <v>41.59</v>
       </c>
-      <c r="G32" s="179"/>
-      <c r="H32" s="179"/>
+      <c r="G32" s="172"/>
+      <c r="H32" s="172"/>
       <c r="I32" s="73">
         <f>B32/D32</f>
         <v>4.4065159505038372</v>
@@ -60199,17 +60199,17 @@
       <c r="A34" s="92">
         <v>1</v>
       </c>
-      <c r="B34" s="178" t="s">
+      <c r="B34" s="171" t="s">
         <v>678</v>
       </c>
-      <c r="C34" s="178"/>
-      <c r="D34" s="178"/>
-      <c r="E34" s="178"/>
-      <c r="F34" s="178"/>
-      <c r="G34" s="178"/>
-      <c r="H34" s="178"/>
-      <c r="I34" s="178"/>
-      <c r="J34" s="178"/>
+      <c r="C34" s="171"/>
+      <c r="D34" s="171"/>
+      <c r="E34" s="171"/>
+      <c r="F34" s="171"/>
+      <c r="G34" s="171"/>
+      <c r="H34" s="171"/>
+      <c r="I34" s="171"/>
+      <c r="J34" s="171"/>
       <c r="L34" s="75"/>
       <c r="M34" s="76"/>
       <c r="N34" s="76"/>
@@ -60237,17 +60237,17 @@
       <c r="A35" s="92">
         <v>2</v>
       </c>
-      <c r="B35" s="178" t="s">
+      <c r="B35" s="171" t="s">
         <v>677</v>
       </c>
-      <c r="C35" s="178"/>
-      <c r="D35" s="178"/>
-      <c r="E35" s="178"/>
-      <c r="F35" s="178"/>
-      <c r="G35" s="178"/>
-      <c r="H35" s="178"/>
-      <c r="I35" s="178"/>
-      <c r="J35" s="178"/>
+      <c r="C35" s="171"/>
+      <c r="D35" s="171"/>
+      <c r="E35" s="171"/>
+      <c r="F35" s="171"/>
+      <c r="G35" s="171"/>
+      <c r="H35" s="171"/>
+      <c r="I35" s="171"/>
+      <c r="J35" s="171"/>
       <c r="L35" s="75"/>
       <c r="M35" s="76"/>
       <c r="N35" s="76"/>
@@ -60264,17 +60264,17 @@
       <c r="A36" s="92">
         <v>3</v>
       </c>
-      <c r="B36" s="178" t="s">
+      <c r="B36" s="171" t="s">
         <v>679</v>
       </c>
-      <c r="C36" s="178"/>
-      <c r="D36" s="178"/>
-      <c r="E36" s="178"/>
-      <c r="F36" s="178"/>
-      <c r="G36" s="178"/>
-      <c r="H36" s="178"/>
-      <c r="I36" s="178"/>
-      <c r="J36" s="178"/>
+      <c r="C36" s="171"/>
+      <c r="D36" s="171"/>
+      <c r="E36" s="171"/>
+      <c r="F36" s="171"/>
+      <c r="G36" s="171"/>
+      <c r="H36" s="171"/>
+      <c r="I36" s="171"/>
+      <c r="J36" s="171"/>
       <c r="L36" s="75"/>
       <c r="M36" s="76"/>
       <c r="N36" s="76"/>
@@ -60291,17 +60291,17 @@
       <c r="A37" s="92">
         <v>4</v>
       </c>
-      <c r="B37" s="178" t="s">
+      <c r="B37" s="171" t="s">
         <v>680</v>
       </c>
-      <c r="C37" s="178"/>
-      <c r="D37" s="178"/>
-      <c r="E37" s="178"/>
-      <c r="F37" s="178"/>
-      <c r="G37" s="178"/>
-      <c r="H37" s="178"/>
-      <c r="I37" s="178"/>
-      <c r="J37" s="178"/>
+      <c r="C37" s="171"/>
+      <c r="D37" s="171"/>
+      <c r="E37" s="171"/>
+      <c r="F37" s="171"/>
+      <c r="G37" s="171"/>
+      <c r="H37" s="171"/>
+      <c r="I37" s="171"/>
+      <c r="J37" s="171"/>
       <c r="L37" s="75"/>
       <c r="M37" s="76"/>
       <c r="N37" s="76"/>
@@ -60318,17 +60318,17 @@
       <c r="A38" s="92">
         <v>5</v>
       </c>
-      <c r="B38" s="178" t="s">
+      <c r="B38" s="171" t="s">
         <v>681</v>
       </c>
-      <c r="C38" s="178"/>
-      <c r="D38" s="178"/>
-      <c r="E38" s="178"/>
-      <c r="F38" s="178"/>
-      <c r="G38" s="178"/>
-      <c r="H38" s="178"/>
-      <c r="I38" s="178"/>
-      <c r="J38" s="178"/>
+      <c r="C38" s="171"/>
+      <c r="D38" s="171"/>
+      <c r="E38" s="171"/>
+      <c r="F38" s="171"/>
+      <c r="G38" s="171"/>
+      <c r="H38" s="171"/>
+      <c r="I38" s="171"/>
+      <c r="J38" s="171"/>
       <c r="L38" s="75"/>
       <c r="M38" s="76"/>
       <c r="N38" s="76"/>
@@ -60640,25 +60640,6 @@
     </row>
   </sheetData>
   <mergeCells count="35">
-    <mergeCell ref="F27:H27"/>
-    <mergeCell ref="F28:H28"/>
-    <mergeCell ref="F29:H29"/>
-    <mergeCell ref="F30:H30"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B38:J38"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F31:H31"/>
-    <mergeCell ref="F32:H32"/>
-    <mergeCell ref="B31:C31"/>
-    <mergeCell ref="B34:J34"/>
-    <mergeCell ref="B35:J35"/>
-    <mergeCell ref="B36:J36"/>
-    <mergeCell ref="B37:J37"/>
     <mergeCell ref="X1:AH1"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
@@ -60675,6 +60656,25 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="A25:J26"/>
+    <mergeCell ref="B38:J38"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F31:H31"/>
+    <mergeCell ref="F32:H32"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B35:J35"/>
+    <mergeCell ref="B36:J36"/>
+    <mergeCell ref="B37:J37"/>
+    <mergeCell ref="F27:H27"/>
+    <mergeCell ref="F28:H28"/>
+    <mergeCell ref="F29:H29"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>